<commit_message>
Friday follow-up run: send Follow-up 4 to 36 due contacts
Final touch in the 5-email sequence for 36 contacts who reached
Follow-up 3 Sent with no response. All replies threaded onto existing
Gmail conversations. Marked Sequence Complete, no bounces/opt-outs/
bookings detected this run.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EVunFkxCQ2WBjC9mX2XzcN
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -4903,11 +4903,11 @@
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G60" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H60" s="5">
         <f>IF(G60="","",TODAY()-G60)</f>
@@ -4915,12 +4915,10 @@
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J60" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J60" s="6" t="n"/>
       <c r="K60" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -4946,7 +4944,7 @@
       </c>
       <c r="R60" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead role at adidas | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead role at adidas | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -4978,11 +4976,11 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G61" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H61" s="5">
         <f>IF(G61="","",TODAY()-G61)</f>
@@ -4990,12 +4988,10 @@
       </c>
       <c r="I61" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J61" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J61" s="6" t="n"/>
       <c r="K61" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -5021,7 +5017,7 @@
       </c>
       <c r="R61" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Manager role at DXC Technology | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Manager role at DXC Technology | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -5053,11 +5049,11 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G62" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H62" s="5">
         <f>IF(G62="","",TODAY()-G62)</f>
@@ -5065,12 +5061,10 @@
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J62" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J62" s="6" t="n"/>
       <c r="K62" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -5096,7 +5090,7 @@
       </c>
       <c r="R62" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales &amp; Business Development Representative role at Zvolv | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Sales &amp; Business Development Representative role at Zvolv | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -5128,11 +5122,11 @@
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G63" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H63" s="5">
         <f>IF(G63="","",TODAY()-G63)</f>
@@ -5140,12 +5134,10 @@
       </c>
       <c r="I63" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J63" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J63" s="6" t="n"/>
       <c r="K63" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -5171,7 +5163,7 @@
       </c>
       <c r="R63" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Business Development Representative - Sales role at TopSource | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Business Development Representative - Sales role at TopSource | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -5203,11 +5195,11 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G64" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H64" s="5">
         <f>IF(G64="","",TODAY()-G64)</f>
@@ -5215,12 +5207,10 @@
       </c>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J64" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J64" s="6" t="n"/>
       <c r="K64" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -5246,7 +5236,7 @@
       </c>
       <c r="R64" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Consultant role at Atos | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Lead Consultant role at Atos | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -5278,11 +5268,11 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G65" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H65" s="5">
         <f>IF(G65="","",TODAY()-G65)</f>
@@ -5290,12 +5280,10 @@
       </c>
       <c r="I65" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J65" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J65" s="6" t="n"/>
       <c r="K65" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -5321,7 +5309,7 @@
       </c>
       <c r="R65" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Consultant role at BT Group | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Lead Consultant role at BT Group | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -5422,11 +5410,11 @@
       </c>
       <c r="F67" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G67" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H67" s="5">
         <f>IF(G67="","",TODAY()-G67)</f>
@@ -5434,12 +5422,10 @@
       </c>
       <c r="I67" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J67" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J67" s="6" t="n"/>
       <c r="K67" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -5465,7 +5451,7 @@
       </c>
       <c r="R67" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Consultant role at Tata Consultancy Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Consultant role at Tata Consultancy Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -5497,11 +5483,11 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G68" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H68" s="5">
         <f>IF(G68="","",TODAY()-G68)</f>
@@ -5509,12 +5495,10 @@
       </c>
       <c r="I68" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J68" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J68" s="6" t="n"/>
       <c r="K68" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -5540,7 +5524,7 @@
       </c>
       <c r="R68" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Consultant - Delivery Lead role at Tata Consultancy Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Consultant - Delivery Lead role at Tata Consultancy Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -5572,11 +5556,11 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G69" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H69" s="5">
         <f>IF(G69="","",TODAY()-G69)</f>
@@ -5584,12 +5568,10 @@
       </c>
       <c r="I69" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J69" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J69" s="6" t="n"/>
       <c r="K69" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -5615,7 +5597,7 @@
       </c>
       <c r="R69" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Consultant role at Northern Trust | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Consultant role at Northern Trust | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -5647,11 +5629,11 @@
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G70" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H70" s="5">
         <f>IF(G70="","",TODAY()-G70)</f>
@@ -5659,12 +5641,10 @@
       </c>
       <c r="I70" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J70" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J70" s="6" t="n"/>
       <c r="K70" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -5690,7 +5670,7 @@
       </c>
       <c r="R70" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Executive role at Capgemini | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Executive role at Capgemini | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -5722,11 +5702,11 @@
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G71" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H71" s="5">
         <f>IF(G71="","",TODAY()-G71)</f>
@@ -5734,12 +5714,10 @@
       </c>
       <c r="I71" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J71" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J71" s="6" t="n"/>
       <c r="K71" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -5765,7 +5743,7 @@
       </c>
       <c r="R71" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Business Development Representative role at Insight | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Business Development Representative role at Insight | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -5797,11 +5775,11 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G72" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H72" s="5">
         <f>IF(G72="","",TODAY()-G72)</f>
@@ -5809,12 +5787,10 @@
       </c>
       <c r="I72" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J72" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J72" s="6" t="n"/>
       <c r="K72" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -5840,7 +5816,7 @@
       </c>
       <c r="R72" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Delivery Consultant role at Vallum Associates | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Lead Delivery Consultant role at Vallum Associates | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -5872,11 +5848,11 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G73" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H73" s="5">
         <f>IF(G73="","",TODAY()-G73)</f>
@@ -5884,12 +5860,10 @@
       </c>
       <c r="I73" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J73" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J73" s="6" t="n"/>
       <c r="K73" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -5915,7 +5889,7 @@
       </c>
       <c r="R73" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Consultant Delivery-Lead role at Worldline Global Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Consultant Delivery-Lead role at Worldline Global Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -6093,11 +6067,11 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G76" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H76" s="5">
         <f>IF(G76="","",TODAY()-G76)</f>
@@ -6105,12 +6079,10 @@
       </c>
       <c r="I76" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J76" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J76" s="6" t="n"/>
       <c r="K76" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -6136,7 +6108,7 @@
       </c>
       <c r="R76" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Delivery Consultant role at LHH | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Lead Delivery Consultant role at LHH | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -6168,11 +6140,11 @@
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G77" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H77" s="5">
         <f>IF(G77="","",TODAY()-G77)</f>
@@ -6180,12 +6152,10 @@
       </c>
       <c r="I77" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J77" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J77" s="6" t="n"/>
       <c r="K77" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -6211,7 +6181,7 @@
       </c>
       <c r="R77" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Delivery Consultant role at Vallum Associates | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Lead Delivery Consultant role at Vallum Associates | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -6312,11 +6282,11 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G79" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H79" s="5">
         <f>IF(G79="","",TODAY()-G79)</f>
@@ -6324,12 +6294,10 @@
       </c>
       <c r="I79" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J79" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J79" s="6" t="n"/>
       <c r="K79" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -6355,7 +6323,7 @@
       </c>
       <c r="R79" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Senior Delivery Manager role at EPAM Systems | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Senior Delivery Manager role at EPAM Systems | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -6387,11 +6355,11 @@
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G80" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H80" s="5">
         <f>IF(G80="","",TODAY()-G80)</f>
@@ -6399,12 +6367,10 @@
       </c>
       <c r="I80" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J80" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J80" s="6" t="n"/>
       <c r="K80" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -6430,7 +6396,7 @@
       </c>
       <c r="R80" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -6746,11 +6712,11 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G85" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H85" s="5">
         <f>IF(G85="","",TODAY()-G85)</f>
@@ -6758,12 +6724,10 @@
       </c>
       <c r="I85" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J85" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J85" s="6" t="n"/>
       <c r="K85" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -6789,7 +6753,7 @@
       </c>
       <c r="R85" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -6890,11 +6854,11 @@
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G87" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H87" s="5">
         <f>IF(G87="","",TODAY()-G87)</f>
@@ -6902,12 +6866,10 @@
       </c>
       <c r="I87" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J87" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J87" s="6" t="n"/>
       <c r="K87" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -6933,7 +6895,7 @@
       </c>
       <c r="R87" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -6965,11 +6927,11 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G88" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H88" s="5">
         <f>IF(G88="","",TODAY()-G88)</f>
@@ -6977,12 +6939,10 @@
       </c>
       <c r="I88" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J88" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J88" s="6" t="n"/>
       <c r="K88" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -7008,7 +6968,7 @@
       </c>
       <c r="R88" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -7040,11 +7000,11 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G89" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H89" s="5">
         <f>IF(G89="","",TODAY()-G89)</f>
@@ -7052,12 +7012,10 @@
       </c>
       <c r="I89" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J89" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J89" s="6" t="n"/>
       <c r="K89" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -7083,7 +7041,7 @@
       </c>
       <c r="R89" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -7115,11 +7073,11 @@
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G90" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H90" s="5">
         <f>IF(G90="","",TODAY()-G90)</f>
@@ -7127,12 +7085,10 @@
       </c>
       <c r="I90" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J90" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J90" s="6" t="n"/>
       <c r="K90" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -7158,7 +7114,7 @@
       </c>
       <c r="R90" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -7267,11 +7223,11 @@
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G92" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H92" s="5">
         <f>IF(G92="","",TODAY()-G92)</f>
@@ -7279,12 +7235,10 @@
       </c>
       <c r="I92" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J92" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J92" s="6" t="n"/>
       <c r="K92" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -7310,7 +7264,7 @@
       </c>
       <c r="R92" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -7419,11 +7373,11 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G94" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H94" s="5">
         <f>IF(G94="","",TODAY()-G94)</f>
@@ -7431,12 +7385,10 @@
       </c>
       <c r="I94" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J94" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J94" s="6" t="n"/>
       <c r="K94" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -7462,7 +7414,7 @@
       </c>
       <c r="R94" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -7494,11 +7446,11 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G95" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H95" s="5">
         <f>IF(G95="","",TODAY()-G95)</f>
@@ -7506,12 +7458,10 @@
       </c>
       <c r="I95" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J95" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J95" s="6" t="n"/>
       <c r="K95" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -7537,7 +7487,7 @@
       </c>
       <c r="R95" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -7569,11 +7519,11 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G96" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H96" s="5">
         <f>IF(G96="","",TODAY()-G96)</f>
@@ -7581,12 +7531,10 @@
       </c>
       <c r="I96" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J96" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J96" s="6" t="n"/>
       <c r="K96" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -7612,7 +7560,7 @@
       </c>
       <c r="R96" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -7644,11 +7592,11 @@
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G97" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H97" s="5">
         <f>IF(G97="","",TODAY()-G97)</f>
@@ -7656,12 +7604,10 @@
       </c>
       <c r="I97" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J97" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J97" s="6" t="n"/>
       <c r="K97" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -7687,7 +7633,7 @@
       </c>
       <c r="R97" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Service Delivery Manager role at V &amp; V Comptech Systems Private Limited | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Service Delivery Manager role at V &amp; V Comptech Systems Private Limited | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -7719,11 +7665,11 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G98" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H98" s="5">
         <f>IF(G98="","",TODAY()-G98)</f>
@@ -7731,12 +7677,10 @@
       </c>
       <c r="I98" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J98" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J98" s="6" t="n"/>
       <c r="K98" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -7762,7 +7706,7 @@
       </c>
       <c r="R98" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -7794,11 +7738,11 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G99" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H99" s="5">
         <f>IF(G99="","",TODAY()-G99)</f>
@@ -7806,12 +7750,10 @@
       </c>
       <c r="I99" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J99" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J99" s="6" t="n"/>
       <c r="K99" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -7837,7 +7779,7 @@
       </c>
       <c r="R99" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -7946,11 +7888,11 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G101" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H101" s="5">
         <f>IF(G101="","",TODAY()-G101)</f>
@@ -7958,12 +7900,10 @@
       </c>
       <c r="I101" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J101" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J101" s="6" t="n"/>
       <c r="K101" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -7989,7 +7929,7 @@
       </c>
       <c r="R101" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -8175,11 +8115,11 @@
       </c>
       <c r="F104" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G104" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H104" s="5">
         <f>IF(G104="","",TODAY()-G104)</f>
@@ -8187,12 +8127,10 @@
       </c>
       <c r="I104" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J104" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J104" s="6" t="n"/>
       <c r="K104" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -8218,7 +8156,7 @@
       </c>
       <c r="R104" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -8250,11 +8188,11 @@
       </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G105" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H105" s="5">
         <f>IF(G105="","",TODAY()-G105)</f>
@@ -8262,12 +8200,10 @@
       </c>
       <c r="I105" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J105" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J105" s="6" t="n"/>
       <c r="K105" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -8293,7 +8229,7 @@
       </c>
       <c r="R105" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -8479,11 +8415,11 @@
       </c>
       <c r="F108" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G108" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H108" s="5">
         <f>IF(G108="","",TODAY()-G108)</f>
@@ -8491,12 +8427,10 @@
       </c>
       <c r="I108" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J108" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J108" s="6" t="n"/>
       <c r="K108" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -8522,7 +8456,7 @@
       </c>
       <c r="R108" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Consultant role at Infosys | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Lead Consultant role at Infosys | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -8554,11 +8488,11 @@
       </c>
       <c r="F109" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G109" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H109" s="5">
         <f>IF(G109="","",TODAY()-G109)</f>
@@ -8566,12 +8500,10 @@
       </c>
       <c r="I109" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J109" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J109" s="6" t="n"/>
       <c r="K109" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -8597,7 +8529,7 @@
       </c>
       <c r="R109" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Manager (Consultant) - Senior Delivery Lead role at Burendo | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Delivery Manager (Consultant) - Senior Delivery Lead role at Burendo | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -8629,11 +8561,11 @@
       </c>
       <c r="F110" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G110" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H110" s="5">
         <f>IF(G110="","",TODAY()-G110)</f>
@@ -8641,12 +8573,10 @@
       </c>
       <c r="I110" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J110" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J110" s="6" t="n"/>
       <c r="K110" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -8672,7 +8602,7 @@
       </c>
       <c r="R110" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Agile Delivery Manager role at tombola | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Agile Delivery Manager role at tombola | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>
@@ -8704,11 +8634,11 @@
       </c>
       <c r="F111" s="5" t="inlineStr">
         <is>
-          <t>Follow-up 3 Sent</t>
+          <t>Sequence Complete</t>
         </is>
       </c>
       <c r="G111" s="6" t="n">
-        <v>46274</v>
+        <v>46276</v>
       </c>
       <c r="H111" s="5">
         <f>IF(G111="","",TODAY()-G111)</f>
@@ -8716,12 +8646,10 @@
       </c>
       <c r="I111" s="5" t="inlineStr">
         <is>
-          <t>Send Follow-up 4</t>
-        </is>
-      </c>
-      <c r="J111" s="6" t="n">
-        <v>46276</v>
-      </c>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="J111" s="6" t="n"/>
       <c r="K111" s="5" t="inlineStr">
         <is>
           <t>N</t>
@@ -8747,7 +8675,7 @@
       </c>
       <c r="R111" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales and Business Development Representative role at Cygnus Group Ltd | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31)</t>
+          <t>Hook: Saw your Sales and Business Development Representative role at Cygnus Group Ltd | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log newsletter announcement broadcast sent to 78 contacts
One-off send announcing the new LinkedIn newsletter post and inviting
existing outreach contacts to subscribe. Excluded Bounced/Opted-Out/
no-email contacts per the permanent exclusion rule. Logged in each
contact's Notes column; Stage/Next Action untouched since this sits
outside the 5-touch sequence.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QpqKsQsMydKcWNEt6cBB1S
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -814,7 +814,7 @@
       </c>
       <c r="R4" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="R5" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -960,7 +960,7 @@
       </c>
       <c r="R6" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="R7" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -1185,7 +1185,7 @@
       </c>
       <c r="R9" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="R10" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Business Development Representative role at REVEL | Renting de Coches</t>
+          <t>Hook: Saw your Sales Business Development Representative role at REVEL | Renting de Coches | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="R11" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1406,7 @@
       </c>
       <c r="R12" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1558,7 @@
       </c>
       <c r="R14" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1631,7 @@
       </c>
       <c r="R15" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -1862,7 +1862,7 @@
       </c>
       <c r="R18" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales Solutions Consultant role at o9 Solutions, Inc.</t>
+          <t>Hook: Saw your Presales Solutions Consultant role at o9 Solutions, Inc. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -2012,7 +2012,7 @@
       </c>
       <c r="R20" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -2162,7 +2162,7 @@
       </c>
       <c r="R22" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -2308,7 +2308,7 @@
       </c>
       <c r="R24" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales Solutions Consultant role at Siemens Digital Industries Software</t>
+          <t>Hook: Saw your Presales Solutions Consultant role at Siemens Digital Industries Software | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -2523,7 +2523,7 @@
       </c>
       <c r="R27" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -2596,7 +2596,7 @@
       </c>
       <c r="R28" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales - Solutions Consultant role at Earnix 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Presales - Solutions Consultant role at Earnix 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -2669,7 +2669,7 @@
       </c>
       <c r="R29" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Solutions Consultant role at ORO Labs 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Solutions Consultant role at ORO Labs 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -2742,7 +2742,7 @@
       </c>
       <c r="R30" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales and Solutions Consultant role at Aspire Systems 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Presales and Solutions Consultant role at Aspire Systems 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -2815,7 +2815,7 @@
       </c>
       <c r="R31" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales &amp; Solutions Consultant role at Columbus 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Presales &amp; Solutions Consultant role at Columbus 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -2965,7 +2965,7 @@
       </c>
       <c r="R33" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales &amp; Solutions Consultant role at Tata Consultancy Services 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Presales &amp; Solutions Consultant role at Tata Consultancy Services 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="R34" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales Solutions Consultant, Bid Manager role at Orange Cyberdefense 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Presales Solutions Consultant, Bid Manager role at Orange Cyberdefense 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="R35" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive Sales Manager role at Haiilo 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Account Executive Sales Manager role at Haiilo 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="R36" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive / Sales Manager role at Storyly 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Account Executive / Sales Manager role at Storyly 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="R37" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive Sales Manager role at TRUE LABS 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Account Executive Sales Manager role at TRUE LABS 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -3330,7 +3330,7 @@
       </c>
       <c r="R38" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive &amp; Sales Manager role at Insure Smart Limited 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Account Executive &amp; Sales Manager role at Insure Smart Limited 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -3403,7 +3403,7 @@
       </c>
       <c r="R39" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager / Account Executive role at CybExer Technologies 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager / Account Executive role at CybExer Technologies 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3476,7 @@
       </c>
       <c r="R40" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales Consultant Manager role at V-Valley 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Presales Consultant Manager role at V-Valley 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -3549,7 +3549,7 @@
       </c>
       <c r="R41" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager, Account Executive role at Alconost 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager, Account Executive role at Alconost 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -3699,7 +3699,7 @@
       </c>
       <c r="R43" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Senior Presales Consultant &amp; Solutions Consultant role at Hexadroit Pvt. Ltd. 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Senior Presales Consultant &amp; Solutions Consultant role at Hexadroit Pvt. Ltd. 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -3849,7 +3849,7 @@
       </c>
       <c r="R45" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Commercial Account Manager role at Boomi 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Commercial Account Manager role at Boomi 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -3922,7 +3922,7 @@
       </c>
       <c r="R46" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager / Account Executive role at yoummday 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager / Account Executive role at yoummday 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -3995,7 +3995,7 @@
       </c>
       <c r="R47" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive / Enterprise Sales role at Neeyamo 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Account Executive / Enterprise Sales role at Neeyamo 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -4214,7 +4214,7 @@
       </c>
       <c r="R50" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager | Account Executive role at kununu 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager | Account Executive role at kununu 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -4287,7 +4287,7 @@
       </c>
       <c r="R51" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager role at Dyad 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager role at Dyad 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -4360,7 +4360,7 @@
       </c>
       <c r="R52" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive | Sales Manager role at Muck Rack 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Account Executive | Sales Manager role at Muck Rack 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -4433,7 +4433,7 @@
       </c>
       <c r="R53" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager - Account Executive role at Arivo 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager - Account Executive role at Arivo 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -4506,7 +4506,7 @@
       </c>
       <c r="R54" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager - Account Executive role at UPTOO 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager - Account Executive role at UPTOO 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -4579,7 +4579,7 @@
       </c>
       <c r="R55" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your SAP Partner Sales Manager &amp; Enterprise Account Executive role at EPI-USE Labs 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your SAP Partner Sales Manager &amp; Enterprise Account Executive role at EPI-USE Labs 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -4652,7 +4652,7 @@
       </c>
       <c r="R56" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager &amp; Account Executive role at Dyad 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager &amp; Account Executive role at Dyad 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -4725,7 +4725,7 @@
       </c>
       <c r="R57" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager / Account Executive role at Tellimer 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager / Account Executive role at Tellimer 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -4798,7 +4798,7 @@
       </c>
       <c r="R58" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Enterprise Account Manager &amp; Sales Manager role at 42Gears 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Enterprise Account Manager &amp; Sales Manager role at 42Gears 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -4871,7 +4871,7 @@
       </c>
       <c r="R59" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Enterprise Sales Manager / Account Executive role at Anakin (YC S21) 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Enterprise Sales Manager / Account Executive role at Anakin (YC S21) 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -4944,7 +4944,7 @@
       </c>
       <c r="R60" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead role at adidas | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead role at adidas | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -5017,7 +5017,7 @@
       </c>
       <c r="R61" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Manager role at DXC Technology | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Manager role at DXC Technology | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5090,7 @@
       </c>
       <c r="R62" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales &amp; Business Development Representative role at Zvolv | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales &amp; Business Development Representative role at Zvolv | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -5163,7 +5163,7 @@
       </c>
       <c r="R63" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Business Development Representative - Sales role at TopSource | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Business Development Representative - Sales role at TopSource | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -5236,7 +5236,7 @@
       </c>
       <c r="R64" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Consultant role at Atos | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Lead Consultant role at Atos | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -5309,7 +5309,7 @@
       </c>
       <c r="R65" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Consultant role at BT Group | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Lead Consultant role at BT Group | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -5451,7 +5451,7 @@
       </c>
       <c r="R67" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Consultant role at Tata Consultancy Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Consultant role at Tata Consultancy Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -5524,7 +5524,7 @@
       </c>
       <c r="R68" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Consultant - Delivery Lead role at Tata Consultancy Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Consultant - Delivery Lead role at Tata Consultancy Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -5597,7 +5597,7 @@
       </c>
       <c r="R69" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Consultant role at Northern Trust | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Consultant role at Northern Trust | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -5670,7 +5670,7 @@
       </c>
       <c r="R70" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Executive role at Capgemini | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Executive role at Capgemini | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -5743,7 +5743,7 @@
       </c>
       <c r="R71" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Business Development Representative role at Insight | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Business Development Representative role at Insight | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -5816,7 +5816,7 @@
       </c>
       <c r="R72" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Delivery Consultant role at Vallum Associates | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Lead Delivery Consultant role at Vallum Associates | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -5889,7 +5889,7 @@
       </c>
       <c r="R73" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Consultant Delivery-Lead role at Worldline Global Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Consultant Delivery-Lead role at Worldline Global Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -6108,7 +6108,7 @@
       </c>
       <c r="R76" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Delivery Consultant role at LHH | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Lead Delivery Consultant role at LHH | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -6181,7 +6181,7 @@
       </c>
       <c r="R77" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Delivery Consultant role at Vallum Associates | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Lead Delivery Consultant role at Vallum Associates | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -6323,7 +6323,7 @@
       </c>
       <c r="R79" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Senior Delivery Manager role at EPAM Systems | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Senior Delivery Manager role at EPAM Systems | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -6396,7 +6396,7 @@
       </c>
       <c r="R80" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -6753,7 +6753,7 @@
       </c>
       <c r="R85" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -6895,7 +6895,7 @@
       </c>
       <c r="R87" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -6968,7 +6968,7 @@
       </c>
       <c r="R88" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -7041,7 +7041,7 @@
       </c>
       <c r="R89" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -7114,7 +7114,7 @@
       </c>
       <c r="R90" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -7264,7 +7264,7 @@
       </c>
       <c r="R92" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -7414,7 +7414,7 @@
       </c>
       <c r="R94" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -7487,7 +7487,7 @@
       </c>
       <c r="R95" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -7560,7 +7560,7 @@
       </c>
       <c r="R96" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -7633,7 +7633,7 @@
       </c>
       <c r="R97" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Service Delivery Manager role at V &amp; V Comptech Systems Private Limited | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Service Delivery Manager role at V &amp; V Comptech Systems Private Limited | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -7706,7 +7706,7 @@
       </c>
       <c r="R98" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -7779,7 +7779,7 @@
       </c>
       <c r="R99" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -7929,7 +7929,7 @@
       </c>
       <c r="R101" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -8156,7 +8156,7 @@
       </c>
       <c r="R104" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -8229,7 +8229,7 @@
       </c>
       <c r="R105" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -8456,7 +8456,7 @@
       </c>
       <c r="R108" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Consultant role at Infosys | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Lead Consultant role at Infosys | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -8529,7 +8529,7 @@
       </c>
       <c r="R109" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Manager (Consultant) - Senior Delivery Lead role at Burendo | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Manager (Consultant) - Senior Delivery Lead role at Burendo | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -8602,7 +8602,7 @@
       </c>
       <c r="R110" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Agile Delivery Manager role at tombola | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Agile Delivery Manager role at tombola | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>
@@ -8675,7 +8675,7 @@
       </c>
       <c r="R111" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales and Business Development Representative role at Cygnus Group Ltd | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales and Business Development Representative role at Cygnus Group Ltd | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter announcement sent 2026-09-25 (LinkedIn newsletter promo: "Demo went perfectly, deal stalled anyway" + subscribe CTA) — one-off broadcast, not part of the 5-touch sequence.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log two stale-sequence bounces from Gmail delivery failures
Bedirhan Akay and Rohit Saha follow-up sends bounced 2026-09-25
(address not found). Both were already Sequence Complete with a
LinkedIn URL, so only Bounced/Bounce Date/Notes were updated per
existing precedent (Stage/Next Action left as-is).

No new leads sourced this run: the Apollo-io connector is
unauthenticated (no tools available), and no manual_sourcing file
matches today's date. See run digest for details, including a
data-integrity finding about an untracked 2026-09-15 send batch.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B6PHG67agGF9P4Qc2wYGLQ
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -949,10 +949,12 @@
       <c r="N6" s="6" t="n"/>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P6" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P6" s="6" t="n">
+        <v>46293</v>
+      </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
           <t>Unknown</t>
@@ -960,7 +962,7 @@
       </c>
       <c r="R6" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Follow-up send bounced 2026-09-25: "Address not found" (mailer-daemon, 550 5.1.1). Sequence was already complete; marking Bounced for the record, no further email to be sent.</t>
         </is>
       </c>
     </row>
@@ -1322,10 +1324,12 @@
       <c r="N11" s="6" t="n"/>
       <c r="O11" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P11" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>46293</v>
+      </c>
       <c r="Q11" s="5" t="inlineStr">
         <is>
           <t>Unknown</t>
@@ -1333,7 +1337,7 @@
       </c>
       <c r="R11" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Follow-up send bounced 2026-09-25: "Address not found" (mailer-daemon). Sequence was already complete; marking Bounced for the record, no further email to be sent.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Friday follow-up run: no sends due, mark 2 bounces detected
No rows in Stage "Follow-up 1 Sent" or "Follow-up 3 Sent" qualified for
Follow-up 2/4 today. Marked Rohit Saha (rohit@ramd.am) and Bedirhan Akay
(bedirhan.akay@apollo.eco) as Bounced=Y after mailer-daemon delivery
failures on 2026-09-25 (both have LinkedIn URLs, so Stage/Next Action
left as-is).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D9NTApxgngKkg9q4YF9eLP
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -949,10 +949,14 @@
       <c r="N6" s="6" t="n"/>
       <c r="O6" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P6" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P6" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
           <t>Unknown</t>
@@ -960,7 +964,7 @@
       </c>
       <c r="R6" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Bounced 2026-09-25: address not found (mailer-daemon), detected via Gmail search on 2026-10-02 (Friday follow-up run). Has LinkedIn URL, left Stage/Next Action as-is.</t>
         </is>
       </c>
     </row>
@@ -1322,10 +1326,14 @@
       <c r="N11" s="6" t="n"/>
       <c r="O11" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="P11" s="6" t="n"/>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P11" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
       <c r="Q11" s="5" t="inlineStr">
         <is>
           <t>Unknown</t>
@@ -1333,7 +1341,7 @@
       </c>
       <c r="R11" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Bounced 2026-09-25: address not found (mailer-daemon), detected via Gmail search on 2026-10-02 (Friday follow-up run). Has LinkedIn URL, left Stage/Next Action as-is.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log newsletter send: article share to 76 active contacts (excl. opted-out/bounced)
One-off content email (not part of the Email1/follow-up cadence) sharing the
"demo mistake" LinkedIn post with every Tracker contact that has a usable
email and is not Opted Out, Bounced, or Booked. Notes column on each of the
76 rows now records the send; Stage/Next Action untouched since this isn't
part of the automated sequence.
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -814,7 +814,7 @@
       </c>
       <c r="R4" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="R5" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="R7" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="R9" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="R10" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Business Development Representative role at REVEL | Renting de Coches</t>
+          <t>Hook: Saw your Sales Business Development Representative role at REVEL | Renting de Coches | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="R12" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -1566,7 +1566,7 @@
       </c>
       <c r="R14" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -1639,7 +1639,7 @@
       </c>
       <c r="R15" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -1870,7 +1870,7 @@
       </c>
       <c r="R18" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales Solutions Consultant role at o9 Solutions, Inc.</t>
+          <t>Hook: Saw your Presales Solutions Consultant role at o9 Solutions, Inc. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
       </c>
       <c r="R20" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2170,7 @@
       </c>
       <c r="R22" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -2316,7 +2316,7 @@
       </c>
       <c r="R24" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales Solutions Consultant role at Siemens Digital Industries Software</t>
+          <t>Hook: Saw your Presales Solutions Consultant role at Siemens Digital Industries Software | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -2531,7 +2531,7 @@
       </c>
       <c r="R27" s="5" t="inlineStr">
         <is>
-          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response.</t>
+          <t>Email 1 sent 2026-08-12 (retroactively logged from Gmail Sent folder — see run digest for context). 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2604,7 @@
       </c>
       <c r="R28" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales - Solutions Consultant role at Earnix 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Presales - Solutions Consultant role at Earnix 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="R29" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Solutions Consultant role at ORO Labs 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Solutions Consultant role at ORO Labs 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -2750,7 +2750,7 @@
       </c>
       <c r="R30" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales and Solutions Consultant role at Aspire Systems 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Presales and Solutions Consultant role at Aspire Systems 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2823,7 @@
       </c>
       <c r="R31" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales &amp; Solutions Consultant role at Columbus 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Presales &amp; Solutions Consultant role at Columbus 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -2973,7 +2973,7 @@
       </c>
       <c r="R33" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales &amp; Solutions Consultant role at Tata Consultancy Services 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Presales &amp; Solutions Consultant role at Tata Consultancy Services 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -3046,7 +3046,7 @@
       </c>
       <c r="R34" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales Solutions Consultant, Bid Manager role at Orange Cyberdefense 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Presales Solutions Consultant, Bid Manager role at Orange Cyberdefense 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -3119,7 +3119,7 @@
       </c>
       <c r="R35" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive Sales Manager role at Haiilo 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Account Executive Sales Manager role at Haiilo 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -3192,7 +3192,7 @@
       </c>
       <c r="R36" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive / Sales Manager role at Storyly 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Account Executive / Sales Manager role at Storyly 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="R37" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive Sales Manager role at TRUE LABS 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Account Executive Sales Manager role at TRUE LABS 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3338,7 @@
       </c>
       <c r="R38" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive &amp; Sales Manager role at Insure Smart Limited 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Account Executive &amp; Sales Manager role at Insure Smart Limited 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="R39" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager / Account Executive role at CybExer Technologies 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager / Account Executive role at CybExer Technologies 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -3484,7 +3484,7 @@
       </c>
       <c r="R40" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Presales Consultant Manager role at V-Valley 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Presales Consultant Manager role at V-Valley 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -3557,7 +3557,7 @@
       </c>
       <c r="R41" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager, Account Executive role at Alconost 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager, Account Executive role at Alconost 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -3707,7 +3707,7 @@
       </c>
       <c r="R43" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Senior Presales Consultant &amp; Solutions Consultant role at Hexadroit Pvt. Ltd. 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Senior Presales Consultant &amp; Solutions Consultant role at Hexadroit Pvt. Ltd. 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -3857,7 +3857,7 @@
       </c>
       <c r="R45" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Commercial Account Manager role at Boomi 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Commercial Account Manager role at Boomi 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -3930,7 +3930,7 @@
       </c>
       <c r="R46" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager / Account Executive role at yoummday 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager / Account Executive role at yoummday 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -4003,7 +4003,7 @@
       </c>
       <c r="R47" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive / Enterprise Sales role at Neeyamo 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Account Executive / Enterprise Sales role at Neeyamo 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -4222,7 +4222,7 @@
       </c>
       <c r="R50" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager | Account Executive role at kununu 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager | Account Executive role at kununu 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -4295,7 +4295,7 @@
       </c>
       <c r="R51" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager role at Dyad 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager role at Dyad 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -4368,7 +4368,7 @@
       </c>
       <c r="R52" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Account Executive | Sales Manager role at Muck Rack 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Account Executive | Sales Manager role at Muck Rack 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -4441,7 +4441,7 @@
       </c>
       <c r="R53" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager - Account Executive role at Arivo 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager - Account Executive role at Arivo 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -4514,7 +4514,7 @@
       </c>
       <c r="R54" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager - Account Executive role at UPTOO 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager - Account Executive role at UPTOO 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       </c>
       <c r="R55" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your SAP Partner Sales Manager &amp; Enterprise Account Executive role at EPI-USE Labs 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your SAP Partner Sales Manager &amp; Enterprise Account Executive role at EPI-USE Labs 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -4660,7 +4660,7 @@
       </c>
       <c r="R56" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager &amp; Account Executive role at Dyad 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager &amp; Account Executive role at Dyad 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -4733,7 +4733,7 @@
       </c>
       <c r="R57" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales Manager / Account Executive role at Tellimer 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales Manager / Account Executive role at Tellimer 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -4806,7 +4806,7 @@
       </c>
       <c r="R58" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Enterprise Account Manager &amp; Sales Manager role at 42Gears 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Enterprise Account Manager &amp; Sales Manager role at 42Gears 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -4879,7 +4879,7 @@
       </c>
       <c r="R59" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Enterprise Sales Manager / Account Executive role at Anakin (YC S21) 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Enterprise Sales Manager / Account Executive role at Anakin (YC S21) 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -4952,7 +4952,7 @@
       </c>
       <c r="R60" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead role at adidas | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead role at adidas | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -5025,7 +5025,7 @@
       </c>
       <c r="R61" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Manager role at DXC Technology | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Manager role at DXC Technology | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -5098,7 +5098,7 @@
       </c>
       <c r="R62" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales &amp; Business Development Representative role at Zvolv | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales &amp; Business Development Representative role at Zvolv | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -5171,7 +5171,7 @@
       </c>
       <c r="R63" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Business Development Representative - Sales role at TopSource | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Business Development Representative - Sales role at TopSource | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -5244,7 +5244,7 @@
       </c>
       <c r="R64" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Consultant role at Atos | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Lead Consultant role at Atos | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -5317,7 +5317,7 @@
       </c>
       <c r="R65" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Consultant role at BT Group | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Lead Consultant role at BT Group | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -5459,7 +5459,7 @@
       </c>
       <c r="R67" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Consultant role at Tata Consultancy Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Consultant role at Tata Consultancy Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5532,7 @@
       </c>
       <c r="R68" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Consultant - Delivery Lead role at Tata Consultancy Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Consultant - Delivery Lead role at Tata Consultancy Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -5605,7 +5605,7 @@
       </c>
       <c r="R69" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Consultant role at Northern Trust | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Consultant role at Northern Trust | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -5678,7 +5678,7 @@
       </c>
       <c r="R70" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Executive role at Capgemini | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Executive role at Capgemini | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -5751,7 +5751,7 @@
       </c>
       <c r="R71" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Business Development Representative role at Insight | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Business Development Representative role at Insight | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -5824,7 +5824,7 @@
       </c>
       <c r="R72" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Delivery Consultant role at Vallum Associates | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Lead Delivery Consultant role at Vallum Associates | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -5897,7 +5897,7 @@
       </c>
       <c r="R73" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Consultant Delivery-Lead role at Worldline Global Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Consultant Delivery-Lead role at Worldline Global Services | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -6116,7 +6116,7 @@
       </c>
       <c r="R76" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Delivery Consultant role at LHH | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Lead Delivery Consultant role at LHH | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -6189,7 +6189,7 @@
       </c>
       <c r="R77" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Delivery Consultant role at Vallum Associates | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Lead Delivery Consultant role at Vallum Associates | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -6331,7 +6331,7 @@
       </c>
       <c r="R79" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Senior Delivery Manager role at EPAM Systems | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Senior Delivery Manager role at EPAM Systems | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -6404,7 +6404,7 @@
       </c>
       <c r="R80" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -6761,7 +6761,7 @@
       </c>
       <c r="R85" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -6903,7 +6903,7 @@
       </c>
       <c r="R87" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -6976,7 +6976,7 @@
       </c>
       <c r="R88" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -7049,7 +7049,7 @@
       </c>
       <c r="R89" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -7122,7 +7122,7 @@
       </c>
       <c r="R90" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -7272,7 +7272,7 @@
       </c>
       <c r="R92" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -7422,7 +7422,7 @@
       </c>
       <c r="R94" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -7495,7 +7495,7 @@
       </c>
       <c r="R95" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -7568,7 +7568,7 @@
       </c>
       <c r="R96" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -7641,7 +7641,7 @@
       </c>
       <c r="R97" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Service Delivery Manager role at V &amp; V Comptech Systems Private Limited | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Service Delivery Manager role at V &amp; V Comptech Systems Private Limited | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -7714,7 +7714,7 @@
       </c>
       <c r="R98" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -7787,7 +7787,7 @@
       </c>
       <c r="R99" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -7937,7 +7937,7 @@
       </c>
       <c r="R101" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -8164,7 +8164,7 @@
       </c>
       <c r="R104" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -8237,7 +8237,7 @@
       </c>
       <c r="R105" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Lead Manager role at Accenture | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -8464,7 +8464,7 @@
       </c>
       <c r="R108" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Lead Consultant role at Infosys | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Lead Consultant role at Infosys | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -8537,7 +8537,7 @@
       </c>
       <c r="R109" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Delivery Manager (Consultant) - Senior Delivery Lead role at Burendo | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Delivery Manager (Consultant) - Senior Delivery Lead role at Burendo | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -8610,7 +8610,7 @@
       </c>
       <c r="R110" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Agile Delivery Manager role at tombola | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Agile Delivery Manager role at tombola | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>
@@ -8683,7 +8683,7 @@
       </c>
       <c r="R111" s="5" t="inlineStr">
         <is>
-          <t>Hook: Saw your Sales and Business Development Representative role at Cygnus Group Ltd | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response.</t>
+          <t>Hook: Saw your Sales and Business Development Representative role at Cygnus Group Ltd | Sourced via Apollo.io web UI (API blocked on abhisri2686 trial plan; manually browsed and exported to Excel 2026-08-31) | 5-touch sequence complete, no response. | Newsletter sent 2026-10-08: demo-trust-framework article (https://lnkd.in/p/ev8ZGf-B).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Send newsletter + subscribe/follow links to 46 new Segment A1 leads
Ad-hoc send of the "AI just did my least favorite part of presales"
LinkedIn article to the 46 of today's 94 newly-added Apollo leads who
have an email address. Each email includes a styled HTML CTA to
subscribe to the LinkedIn newsletter and a link to follow Abhineet's
LinkedIn profile, alongside a plain-text fallback. Logged to each
affected Tracker row's Notes for audit trail; Stage/Next Action left
untouched since this is independent of the formal cold-outreach Email 1
cadence, which remains queued for these contacts.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NVjtpTpeX4sJP8Cb5MAHV2
</commit_message>
<xml_diff>
--- a/tracker.xlsx
+++ b/tracker.xlsx
@@ -8725,7 +8725,7 @@
       </c>
       <c r="R112" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at HCLTech | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 234000</t>
+          <t>Saw your Presales Consultant role at HCLTech | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 234000 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -8798,7 +8798,7 @@
       </c>
       <c r="R113" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at HCLTech | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 234000</t>
+          <t>Saw your Presales Consultant role at HCLTech | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 234000 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -8871,7 +8871,7 @@
       </c>
       <c r="R114" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at HCLTech | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 234000</t>
+          <t>Saw your Presales Consultant role at HCLTech | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 234000 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -8944,7 +8944,7 @@
       </c>
       <c r="R115" s="18" t="inlineStr">
         <is>
-          <t>Saw your PreSales Consultant role at Team Computers | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 5500</t>
+          <t>Saw your PreSales Consultant role at Team Computers | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 5500 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -9017,7 +9017,7 @@
       </c>
       <c r="R116" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Indictrans | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 100</t>
+          <t>Saw your Presales Consultant role at Indictrans | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 100 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -9090,7 +9090,7 @@
       </c>
       <c r="R117" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Infosys | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 328000</t>
+          <t>Saw your Presales Consultant role at Infosys | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 328000 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -9163,7 +9163,7 @@
       </c>
       <c r="R118" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Accenture | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 799000</t>
+          <t>Saw your Presales Consultant role at Accenture | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 799000 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -9374,7 +9374,7 @@
       </c>
       <c r="R121" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at MetricStream | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 1300</t>
+          <t>Saw your Presales Consultant role at MetricStream | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 1300 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -9447,7 +9447,7 @@
       </c>
       <c r="R122" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Nagarro | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 19000</t>
+          <t>Saw your Presales Consultant role at Nagarro | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 19000 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -9520,7 +9520,7 @@
       </c>
       <c r="R123" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Eastern Software Solutions | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 630</t>
+          <t>Saw your Presales Consultant role at Eastern Software Solutions | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 630 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -9593,7 +9593,7 @@
       </c>
       <c r="R124" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Cognizant | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 357000</t>
+          <t>Saw your Presales Consultant role at Cognizant | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 357000 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -9666,7 +9666,7 @@
       </c>
       <c r="R125" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Sotiotech | Go-To ServiceNow Partner | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 49</t>
+          <t>Saw your Presales Consultant role at Sotiotech | Go-To ServiceNow Partner | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 49 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -9739,7 +9739,7 @@
       </c>
       <c r="R126" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Veefin | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 290</t>
+          <t>Saw your Presales Consultant role at Veefin | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 290 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -9812,7 +9812,7 @@
       </c>
       <c r="R127" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Valuehub | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 180</t>
+          <t>Saw your Presales Consultant role at Valuehub | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 180 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -9885,7 +9885,7 @@
       </c>
       <c r="R128" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Tecnotree Corporation | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 760</t>
+          <t>Saw your Presales Consultant role at Tecnotree Corporation | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 760 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -9958,7 +9958,7 @@
       </c>
       <c r="R129" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Cyfuture | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 5000</t>
+          <t>Saw your Presales Consultant role at Cyfuture | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 5000 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -10031,7 +10031,7 @@
       </c>
       <c r="R130" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Autoplant System India Pvt. Ltd. | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 350</t>
+          <t>Saw your Presales Consultant role at Autoplant System India Pvt. Ltd. | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 350 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -10104,7 +10104,7 @@
       </c>
       <c r="R131" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at L&amp;T Technology Services | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 22000</t>
+          <t>Saw your Presales Consultant role at L&amp;T Technology Services | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 22000 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -10177,7 +10177,7 @@
       </c>
       <c r="R132" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Autoplant System India Pvt. Ltd. | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 350</t>
+          <t>Saw your Presales Consultant role at Autoplant System India Pvt. Ltd. | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 350 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -10250,7 +10250,7 @@
       </c>
       <c r="R133" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Execo | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 500</t>
+          <t>Saw your Presales Consultant role at Execo | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 500 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -10323,7 +10323,7 @@
       </c>
       <c r="R134" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at qBotica | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 200</t>
+          <t>Saw your Presales Consultant role at qBotica | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 200 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -10396,7 +10396,7 @@
       </c>
       <c r="R135" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at HCLTech | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 234000</t>
+          <t>Saw your Presales Consultant role at HCLTech | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 234000 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -10469,7 +10469,7 @@
       </c>
       <c r="R136" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at PTR Global | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 260</t>
+          <t>Saw your Presales Consultant role at PTR Global | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 260 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -10542,7 +10542,7 @@
       </c>
       <c r="R137" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Vast Edge Cloud Backup, Apps | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 60</t>
+          <t>Saw your Presales Consultant role at Vast Edge Cloud Backup, Apps | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 60 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -10615,7 +10615,7 @@
       </c>
       <c r="R138" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Wipro | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 240000</t>
+          <t>Saw your Presales Consultant role at Wipro | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 240000 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -10688,7 +10688,7 @@
       </c>
       <c r="R139" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Wipro | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 240000</t>
+          <t>Saw your Presales Consultant role at Wipro | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 240000 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -10761,7 +10761,7 @@
       </c>
       <c r="R140" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Solytics Partners | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 430</t>
+          <t>Saw your Presales Consultant role at Solytics Partners | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 430 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -10834,7 +10834,7 @@
       </c>
       <c r="R141" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Infojini Inc | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 950</t>
+          <t>Saw your Presales Consultant role at Infojini Inc | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 950 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -10976,7 +10976,7 @@
       </c>
       <c r="R143" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Capgemini | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 423000</t>
+          <t>Saw your Presales Consultant role at Capgemini | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 423000 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -11049,7 +11049,7 @@
       </c>
       <c r="R144" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Wipro | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 240000</t>
+          <t>Saw your Presales Consultant role at Wipro | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 240000 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -11122,7 +11122,7 @@
       </c>
       <c r="R145" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at HCLTech | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 234000</t>
+          <t>Saw your Presales Consultant role at HCLTech | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 234000 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -11195,7 +11195,7 @@
       </c>
       <c r="R146" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Genpact | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 141000</t>
+          <t>Saw your Presales Consultant role at Genpact | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 141000 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -11268,7 +11268,7 @@
       </c>
       <c r="R147" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Swan Solutions &amp; Services Pvt Ltd. | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 250</t>
+          <t>Saw your Presales Consultant role at Swan Solutions &amp; Services Pvt Ltd. | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 250 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -11341,7 +11341,7 @@
       </c>
       <c r="R148" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Solytics Partners | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 430</t>
+          <t>Saw your Presales Consultant role at Solytics Partners | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 430 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -11414,7 +11414,7 @@
       </c>
       <c r="R149" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Prospecta Software | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 380</t>
+          <t>Saw your Presales Consultant role at Prospecta Software | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 380 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -11487,7 +11487,7 @@
       </c>
       <c r="R150" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Incite Gravity | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 38</t>
+          <t>Saw your Presales Consultant role at Incite Gravity | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 38 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -11560,7 +11560,7 @@
       </c>
       <c r="R151" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Genzeon | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 670</t>
+          <t>Saw your Presales Consultant role at Genzeon | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 670 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -11633,7 +11633,7 @@
       </c>
       <c r="R152" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at eWorkplace Apps | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 75</t>
+          <t>Saw your Presales Consultant role at eWorkplace Apps | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 75 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -11706,7 +11706,7 @@
       </c>
       <c r="R153" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Photon | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 7500</t>
+          <t>Saw your Presales Consultant role at Photon | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 7500 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -11779,7 +11779,7 @@
       </c>
       <c r="R154" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at Thinkinnov Solution Technologies Private Limited | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 120</t>
+          <t>Saw your Presales Consultant role at Thinkinnov Solution Technologies Private Limited | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 120 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -11852,7 +11852,7 @@
       </c>
       <c r="R155" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at iONE IT Solutions Pvt. Ltd. | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 62</t>
+          <t>Saw your Presales Consultant role at iONE IT Solutions Pvt. Ltd. | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 62 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -14616,7 +14616,7 @@
       </c>
       <c r="R195" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at AlphaSense | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 3800</t>
+          <t>Saw your Presales Consultant role at AlphaSense | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 3800 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -14689,7 +14689,7 @@
       </c>
       <c r="R196" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at M.Tech | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 600</t>
+          <t>Saw your Presales Consultant role at M.Tech | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 600 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -14762,7 +14762,7 @@
       </c>
       <c r="R197" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at AvePoint | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 3500</t>
+          <t>Saw your Presales Consultant role at AvePoint | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 3500 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -14835,7 +14835,7 @@
       </c>
       <c r="R198" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at QuantHouse | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 87</t>
+          <t>Saw your Presales Consultant role at QuantHouse | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 87 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -14908,7 +14908,7 @@
       </c>
       <c r="R199" s="18" t="inlineStr">
         <is>
-          <t>Saw your Presales Consultant role at BigObject Inc. | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 28</t>
+          <t>Saw your Presales Consultant role at BigObject Inc. | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 28 | Newsletter sent 2026-10-23: "AI just did my least favorite part of presales" (LinkedIn article), with newsletter-subscribe and profile-follow links included.</t>
         </is>
       </c>
     </row>
@@ -14982,36 +14982,36 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" t="inlineStr">
+      <c r="A201" s="11" t="inlineStr">
         <is>
           <t>Geoffrey Hernandez</t>
         </is>
       </c>
-      <c r="C201" t="inlineStr">
+      <c r="C201" s="11" t="inlineStr">
         <is>
           <t>http://www.linkedin.com/in/geoffrey-h-99602123</t>
         </is>
       </c>
-      <c r="D201" t="inlineStr">
+      <c r="D201" s="11" t="inlineStr">
         <is>
           <t>Apollo.io</t>
         </is>
       </c>
-      <c r="E201" t="inlineStr">
+      <c r="E201" s="11" t="inlineStr">
         <is>
           <t>Sales &amp; Presales Career Progression</t>
         </is>
       </c>
-      <c r="F201" t="inlineStr">
+      <c r="F201" s="11" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="H201">
+      <c r="H201" s="11">
         <f>IF(G201="","",TODAY()-G201)</f>
         <v/>
       </c>
-      <c r="I201" t="inlineStr">
+      <c r="I201" s="11" t="inlineStr">
         <is>
           <t>Send LinkedIn Connection Request</t>
         </is>
@@ -15019,63 +15019,63 @@
       <c r="J201" s="23" t="n">
         <v>46318</v>
       </c>
-      <c r="K201" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M201" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O201" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q201" t="inlineStr">
+      <c r="K201" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M201" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O201" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q201" s="11" t="inlineStr">
         <is>
           <t>Singapore</t>
         </is>
       </c>
-      <c r="R201" t="inlineStr">
+      <c r="R201" s="11" t="inlineStr">
         <is>
           <t>Saw your Presales Consultant role at Crayon | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 2700</t>
         </is>
       </c>
     </row>
     <row r="202">
-      <c r="A202" t="inlineStr">
+      <c r="A202" s="11" t="inlineStr">
         <is>
           <t>Pulkit Agarwal</t>
         </is>
       </c>
-      <c r="C202" t="inlineStr">
+      <c r="C202" s="11" t="inlineStr">
         <is>
           <t>http://www.linkedin.com/in/pulkit4501</t>
         </is>
       </c>
-      <c r="D202" t="inlineStr">
+      <c r="D202" s="11" t="inlineStr">
         <is>
           <t>Apollo.io</t>
         </is>
       </c>
-      <c r="E202" t="inlineStr">
+      <c r="E202" s="11" t="inlineStr">
         <is>
           <t>Sales &amp; Presales Career Progression</t>
         </is>
       </c>
-      <c r="F202" t="inlineStr">
+      <c r="F202" s="11" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="H202">
+      <c r="H202" s="11">
         <f>IF(G202="","",TODAY()-G202)</f>
         <v/>
       </c>
-      <c r="I202" t="inlineStr">
+      <c r="I202" s="11" t="inlineStr">
         <is>
           <t>Send LinkedIn Connection Request</t>
         </is>
@@ -15083,63 +15083,63 @@
       <c r="J202" s="23" t="n">
         <v>46318</v>
       </c>
-      <c r="K202" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M202" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O202" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q202" t="inlineStr">
+      <c r="K202" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M202" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O202" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q202" s="11" t="inlineStr">
         <is>
           <t>Singapore</t>
         </is>
       </c>
-      <c r="R202" t="inlineStr">
+      <c r="R202" s="11" t="inlineStr">
         <is>
           <t>Saw your Presales Consultant role at Slimstock | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 600</t>
         </is>
       </c>
     </row>
     <row r="203">
-      <c r="A203" t="inlineStr">
+      <c r="A203" s="11" t="inlineStr">
         <is>
           <t>Juan Teo</t>
         </is>
       </c>
-      <c r="C203" t="inlineStr">
+      <c r="C203" s="11" t="inlineStr">
         <is>
           <t>http://www.linkedin.com/in/teojuansiew</t>
         </is>
       </c>
-      <c r="D203" t="inlineStr">
+      <c r="D203" s="11" t="inlineStr">
         <is>
           <t>Apollo.io</t>
         </is>
       </c>
-      <c r="E203" t="inlineStr">
+      <c r="E203" s="11" t="inlineStr">
         <is>
           <t>Sales &amp; Presales Career Progression</t>
         </is>
       </c>
-      <c r="F203" t="inlineStr">
+      <c r="F203" s="11" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="H203">
+      <c r="H203" s="11">
         <f>IF(G203="","",TODAY()-G203)</f>
         <v/>
       </c>
-      <c r="I203" t="inlineStr">
+      <c r="I203" s="11" t="inlineStr">
         <is>
           <t>Send LinkedIn Connection Request</t>
         </is>
@@ -15147,63 +15147,63 @@
       <c r="J203" s="23" t="n">
         <v>46318</v>
       </c>
-      <c r="K203" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M203" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O203" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q203" t="inlineStr">
+      <c r="K203" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M203" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O203" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q203" s="11" t="inlineStr">
         <is>
           <t>Singapore</t>
         </is>
       </c>
-      <c r="R203" t="inlineStr">
+      <c r="R203" s="11" t="inlineStr">
         <is>
           <t>Saw your Presales Consultant role at Elixir Technology | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 51</t>
         </is>
       </c>
     </row>
     <row r="204">
-      <c r="A204" t="inlineStr">
+      <c r="A204" s="11" t="inlineStr">
         <is>
           <t>Sibikrishnan</t>
         </is>
       </c>
-      <c r="C204" t="inlineStr">
+      <c r="C204" s="11" t="inlineStr">
         <is>
           <t>http://www.linkedin.com/in/agsibikrishnan</t>
         </is>
       </c>
-      <c r="D204" t="inlineStr">
+      <c r="D204" s="11" t="inlineStr">
         <is>
           <t>Apollo.io</t>
         </is>
       </c>
-      <c r="E204" t="inlineStr">
+      <c r="E204" s="11" t="inlineStr">
         <is>
           <t>Sales &amp; Presales Career Progression</t>
         </is>
       </c>
-      <c r="F204" t="inlineStr">
+      <c r="F204" s="11" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="H204">
+      <c r="H204" s="11">
         <f>IF(G204="","",TODAY()-G204)</f>
         <v/>
       </c>
-      <c r="I204" t="inlineStr">
+      <c r="I204" s="11" t="inlineStr">
         <is>
           <t>Send LinkedIn Connection Request</t>
         </is>
@@ -15211,63 +15211,63 @@
       <c r="J204" s="23" t="n">
         <v>46318</v>
       </c>
-      <c r="K204" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M204" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O204" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q204" t="inlineStr">
+      <c r="K204" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M204" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O204" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q204" s="11" t="inlineStr">
         <is>
           <t>Singapore</t>
         </is>
       </c>
-      <c r="R204" t="inlineStr">
+      <c r="R204" s="11" t="inlineStr">
         <is>
           <t>Saw your Presales Consultant role at Jeen.ai | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 140</t>
         </is>
       </c>
     </row>
     <row r="205">
-      <c r="A205" t="inlineStr">
+      <c r="A205" s="11" t="inlineStr">
         <is>
           <t>Betty Jiun</t>
         </is>
       </c>
-      <c r="C205" t="inlineStr">
+      <c r="C205" s="11" t="inlineStr">
         <is>
           <t>http://www.linkedin.com/in/betty-tan-rou-jiun-21369b137</t>
         </is>
       </c>
-      <c r="D205" t="inlineStr">
+      <c r="D205" s="11" t="inlineStr">
         <is>
           <t>Apollo.io</t>
         </is>
       </c>
-      <c r="E205" t="inlineStr">
+      <c r="E205" s="11" t="inlineStr">
         <is>
           <t>Sales &amp; Presales Career Progression</t>
         </is>
       </c>
-      <c r="F205" t="inlineStr">
+      <c r="F205" s="11" t="inlineStr">
         <is>
           <t>New</t>
         </is>
       </c>
-      <c r="H205">
+      <c r="H205" s="11">
         <f>IF(G205="","",TODAY()-G205)</f>
         <v/>
       </c>
-      <c r="I205" t="inlineStr">
+      <c r="I205" s="11" t="inlineStr">
         <is>
           <t>Send LinkedIn Connection Request</t>
         </is>
@@ -15275,27 +15275,27 @@
       <c r="J205" s="23" t="n">
         <v>46318</v>
       </c>
-      <c r="K205" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="M205" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O205" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q205" t="inlineStr">
+      <c r="K205" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M205" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O205" s="11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q205" s="11" t="inlineStr">
         <is>
           <t>Singapore</t>
         </is>
       </c>
-      <c r="R205" t="inlineStr">
+      <c r="R205" s="11" t="inlineStr">
         <is>
           <t>Saw your Presales Consultant role at 1CLOUDSTAR | Sourced via Apollo.io web UI (manual export; expanded geography incl. US/UK/Australia/Canada per Abhineet's 2026-10-23 approval) | Company size: 19</t>
         </is>

</xml_diff>